<commit_message>
Update REST/MQTT examples from live review and cloudConfig set.
Refresh endpoint packs, Excel tracking, and rebuilt OpenAPI; add cloudConfig all-channel and data-transport examples.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/FXR90-Examples-Effort-Effectiveness.xlsx
+++ b/FXR90-Examples-Effort-Effectiveness.xlsx
@@ -525,7 +525,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="199.95" customHeight="1" s="12">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -552,7 +551,6 @@
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -632,11 +630,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
@@ -672,11 +665,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
@@ -712,20 +700,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
@@ -733,25 +707,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
@@ -759,30 +714,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
@@ -790,35 +721,6 @@
         </is>
       </c>
     </row>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
@@ -1005,7 +907,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>SPEC DEFECT: GPIO-LED oneOf is string-only; in-spec {} example is invalid; Has 1 response example ((inline)); Ready in grok-examples: +0 request, +1 response PROPOSED file(s)</t>
+          <t>DEFERRED — do later. Finalize a good GET setting example after PUT settles.</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
@@ -1032,12 +934,17 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Fix schema, then keep/adjust examples</t>
+          <t>Deferred — do later</t>
         </is>
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-config/GET/response.200.gpio_led_not_configured.json</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Deferred — do later (good setting)</t>
         </is>
       </c>
     </row>
@@ -1082,7 +989,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>SPEC DEFECT: IPV6.prefix typed string but examples use integer 64; Has 5 response examples — good coverage</t>
+          <t>UPDATED per Krishna: wan0 not supported on FXR60 — WAN examples marked FXR90 only.</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
@@ -1109,12 +1016,17 @@
       </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>Fix schema, then keep/adjust examples</t>
+          <t>Reviewed — wan0 FXR90 only (Krishna)</t>
         </is>
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Updated — wan0 not on FXR60</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1071,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>SPEC DEFECT: IPV6.prefix typed string but examples use integer 64; Has 17 named request examples — good coverage; Response is empty-string on success; no example (low value)</t>
+          <t>UPDATED per Krishna: wan0 not supported on FXR60 — WAN examples marked FXR90 only.</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
@@ -1186,12 +1098,17 @@
       </c>
       <c r="P7" s="4" t="inlineStr">
         <is>
-          <t>Fix schema, then keep/adjust examples</t>
+          <t>Reviewed — wan0 FXR90 only (Krishna)</t>
         </is>
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Updated — wan0 not on FXR60</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1153,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: GET examples DEFAULT/NON_DEFAULT. Folder: reviewed-by-me/cloud-app-led/GET/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
@@ -1263,7 +1180,7 @@
       </c>
       <c r="P8" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — GET examples approved in reviewed-by-me/cloud-app-led/GET/</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q8" s="4" t="inlineStr">
@@ -1273,7 +1190,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-app-led/ (GET)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1235,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET response example (gpi_status). Summary: Current GPI pin states. Folder: reviewed-by-me/cloud-gpi/. Also in FXR60-90 rest/operation_examples + mqtt/examples/get_gpi_status.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
@@ -1345,7 +1262,7 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — one GET example (gpi_status) approved; merge into canonical YAML when asked</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
@@ -1355,7 +1272,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-gpi/ (gpi_status)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1317,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET response example (gpo_status). Summary: Current GPO pin states. Folder: reviewed-by-me/cloud-gpo/. Also in FXR60-90 rest/operation_examples + mqtt/examples/get_gpostatus. Applies To set to FXR60 / FXR90.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
@@ -1427,7 +1344,7 @@
       </c>
       <c r="P10" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — one GET example (gpo_status) approved; merge into canonical YAML when asked</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q10" s="4" t="inlineStr">
@@ -1437,7 +1354,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-gpo/ (gpo_status)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1399,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>MISSING response example (schema declares JSON); Ready in grok-examples: +0 request, +1 response PROPOSED file(s)</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
@@ -1509,7 +1426,7 @@
       </c>
       <c r="P11" s="4" t="inlineStr">
         <is>
-          <t>Deferred — focus later</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q11" s="4" t="inlineStr">
@@ -1519,7 +1436,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Deferred — focus later</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1481,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET response example (login_success). Summary: Bearer token returned. Folder: reviewed-by-me/cloud-localrestlogin/. REST-only (no MQTT).</t>
+          <t>UPDATED by review: login_success approved on live reader.</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
@@ -1591,7 +1508,7 @@
       </c>
       <c r="P12" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — one GET example (login_success) approved; merge into canonical YAML when asked</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q12" s="4" t="inlineStr">
@@ -1601,7 +1518,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-localrestlogin/ (login_success)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1563,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET response example (ntp_server). Summary: Current NTP server. Folder: reviewed-by-me/cloud-ntpserver/.</t>
+          <t>DISCUSS with Mayur / Dhavnesh before finalizing examples.</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
@@ -1673,7 +1590,7 @@
       </c>
       <c r="P13" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — one GET example (ntp_server) approved; merge into canonical YAML when asked</t>
+          <t>Discuss with Mayur/Dhavnesh</t>
         </is>
       </c>
       <c r="Q13" s="4" t="inlineStr">
@@ -1683,7 +1600,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-ntpserver/ (ntp_server)</t>
+          <t>Discuss with Mayur/Dhavnesh</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1645,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET example (pre_selection). Summary: Current preSelection state. NOTE — discuss with developer: GET returns string enabled/disabled, but PUT uses boolean true/false. Confirm intended contract before docs merge.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
@@ -1755,7 +1672,7 @@
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — example OK. Discuss with developer: GET string vs PUT boolean mismatch.</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q14" s="4" t="inlineStr">
@@ -1765,7 +1682,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-preselection/ (pre_selection) — discuss GET/PUT types with developer</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1809,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — focus later (FXR60 only; not on FXR90 — use app-led). GET and PUT both deferred together.</t>
+          <t>DISCUSS WITH QA — known issue on GET/PUT stack-led (FXR60).</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
@@ -1919,7 +1836,7 @@
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>Deferred — focus later (FXR60 only)</t>
+          <t>Discuss with QA</t>
         </is>
       </c>
       <c r="Q16" s="4" t="inlineStr">
@@ -1929,7 +1846,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Deferred — focus later</t>
+          <t>Discuss with QA — GET/PUT stack-led</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1891,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET response example (time_zone). Summary: Current time zone. Folder: reviewed-by-me/cloud-timezone/. Optional discuss with developer: GET long-form vs PUT short-form zone strings.</t>
+          <t>UPDATED by review: GET example time_zone = UTC.</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
@@ -2001,7 +1918,7 @@
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — one GET example (time_zone) approved; merge into canonical YAML when asked</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
@@ -2011,7 +1928,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-timezone/ (time_zone)</t>
+          <t>Updated — time_zone UTC</t>
         </is>
       </c>
     </row>
@@ -2056,7 +1973,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request (app_led) — Amber blink for 60 seconds. Response example added: success = empty string. NEED LIVE TEST: run PUT on a reader and confirm 200 body is really empty string (Swagger used to show placeholder 'string'). Folder: reviewed-by-me/cloud-app-led/PUT/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
@@ -2083,7 +2000,7 @@
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — examples ready. NEED LIVE TEST to confirm empty-string success response</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
@@ -2093,7 +2010,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-app-led/ (app_led) — NEED LIVE TEST for response</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2055,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: DELETE response success = empty string. Path caname example AmazonRootCA1. NEED LIVE TEST: confirm delete uses path {caname} only (no body name field). Folder: reviewed-by-me/cloud-cacertificates-caname/DELETE/.</t>
+          <t>DISCUSS with Mayur — GET/PUT/DELETE caCertificates.</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
@@ -2165,7 +2082,7 @@
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — DELETE success ready. NEED LIVE TEST: name in path vs body</t>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
       <c r="Q19" s="4" t="inlineStr">
@@ -2175,7 +2092,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-cacertificates-caname/ (success) — NEED LIVE TEST path vs name</t>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2137,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request cable_loss — Port 1: 90 ft at 18 dB/100ft. Response success = empty string. Folder: reviewed-by-me/cloud-cablelosscompensation/PUT/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
@@ -2247,7 +2164,7 @@
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — examples ready</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q20" s="4" t="inlineStr">
@@ -2257,7 +2174,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-cablelosscompensation/ (cable_loss)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2219,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET example installed — Server and client certificates. NEED LIVE TEST: confirm real reader returns this shape (name/type/serial/validity/publickey) and field names match. Folder: reviewed-by-me/cloud-certificates/GET/.</t>
+          <t>UPDATED by review: live certificate list (client COMMON + server).</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
@@ -2329,7 +2246,7 @@
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — installed ready. NEED LIVE TEST against reader response shape</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q21" s="4" t="inlineStr">
@@ -2339,7 +2256,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-certificates/ (installed) — NEED LIVE TEST</t>
+          <t>Updated — live installed certificates</t>
         </is>
       </c>
     </row>
@@ -2384,7 +2301,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: DELETE success empty string; path certname=mqtt-client-cert; query type=client. MQTT del_certs payload name+type. Removed invalid server/misnamed examples. Folder: reviewed-by-me/cloud-certificates-certname/DELETE/.</t>
+          <t>DISCUSS WITH QA — do we need type as a parameter on DELETE?</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
@@ -2411,7 +2328,7 @@
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — DELETE + MQTT del_certs ready</t>
+          <t>Discuss with QA — type parameter?</t>
         </is>
       </c>
       <c r="Q22" s="4" t="inlineStr">
@@ -2421,7 +2338,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-certificates-certname/ (success) + mqtt del_certs</t>
+          <t>Discuss with QA — type on DELETE?</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2383,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single GET example profiles_present — Two profiles. Removed no_profiles. Folder: reviewed-by-me/cloud-esimconfig/GET/.</t>
+          <t>UPDATED by review: Applies To FXR90 only (not FXR60).</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
@@ -2493,7 +2410,7 @@
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — single GET example ready</t>
+          <t>Reviewed — FXR90 only</t>
         </is>
       </c>
       <c r="Q23" s="4" t="inlineStr">
@@ -2503,7 +2420,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-esimconfig/ (profiles_present)</t>
+          <t>Updated — FXR90 only</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2465,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request gpo — Port 3 HIGH. Response success = empty string. Removed port1_high and port3_low. Folder: reviewed-by-me/cloud-gpo/PUT/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
@@ -2575,7 +2492,7 @@
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — single PUT example ready</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q24" s="4" t="inlineStr">
@@ -2585,7 +2502,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-gpo/ (gpo)</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2547,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — focus later (with GET hostName). Open questions: RFC lowercase hostname vs serial-style sample; GET field hostName vs PUT key hostname casing. Draft packs: hostName.json / hostName_lab.json.</t>
+          <t>UPDATED by review: single PUT example (hostName). Removed second lab example.</t>
         </is>
       </c>
       <c r="J25" s="4" t="n">
@@ -2657,7 +2574,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>Deferred — focus later (with GET hostName)</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
@@ -2667,7 +2584,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Deferred — focus later</t>
+          <t>Updated — one hostName example</t>
         </is>
       </c>
     </row>
@@ -3204,7 +3121,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request pre_selection — Enable preSelection (true). Response success = empty string. Removed enable/disable duplicates. NEED LIVE TEST: PUT boolean vs GET string enabled/disabled. Folder: reviewed-by-me/cloud-preselection/PUT/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J32" s="4" t="n">
@@ -3231,7 +3148,7 @@
       </c>
       <c r="P32" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — example ready. NEED LIVE TEST boolean vs GET string</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q32" s="4" t="inlineStr">
@@ -3241,7 +3158,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-preselection/ (pre_selection) — NEED LIVE TEST</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -3286,7 +3203,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: response success = empty string; no request body. NEED LIVE TEST: confirm empty-string success before disconnect (disruptive). Folder: reviewed-by-me/cloud-reboot/PUT/.</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
@@ -3313,7 +3230,7 @@
       </c>
       <c r="P33" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — example ready. NEED LIVE TEST (reboot disruptive)</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q33" s="4" t="inlineStr">
@@ -3323,7 +3240,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-reboot/ (success) — NEED LIVE TEST</t>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3285,7 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request region — USA FCC Part 15.247. Response success = empty string. Removed Canada/India variants. NEED LIVE TEST: confirm against supportedRegionList/supportedStandardList. Folder: reviewed-by-me/cloud-region/PUT/.</t>
+          <t>UPDATED by review: single PUT example (region) — Canada / CANADA_FCC_15.</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
@@ -3395,7 +3312,7 @@
       </c>
       <c r="P34" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — example ready. NEED LIVE TEST against supported lists</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q34" s="4" t="inlineStr">
@@ -3405,7 +3322,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-region/ (region) — NEED LIVE TEST</t>
+          <t>Updated — one region PUT (Canada)</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3367,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — focus later (FXR60 only; not on FXR90 — use app-led). GET and PUT both deferred together.</t>
+          <t>DISCUSS WITH QA — known issue on GET/PUT stack-led (FXR60).</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
@@ -3477,7 +3394,7 @@
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
-          <t>Deferred — focus later (FXR60 only)</t>
+          <t>Discuss with QA</t>
         </is>
       </c>
       <c r="Q35" s="4" t="inlineStr">
@@ -3487,7 +3404,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Deferred — focus later</t>
+          <t>Discuss with QA — GET/PUT stack-led</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3449,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT request time_zone — Set time zone UTC. Response success = empty string. Removed Kolkata/UTC duplicates. NEED LIVE TEST: short PUT name vs long GET display string. Folder: reviewed-by-me/cloud-timezone/PUT/.</t>
+          <t>UPDATED by review: two PUT examples from enum — UTC and Kolkata.</t>
         </is>
       </c>
       <c r="J36" s="4" t="n">
@@ -3559,7 +3476,7 @@
       </c>
       <c r="P36" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — example ready. NEED LIVE TEST short vs long names</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q36" s="4" t="inlineStr">
@@ -3569,7 +3486,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Updated — reviewed-by-me/cloud-timezone/ (time_zone) — NEED LIVE TEST</t>
+          <t>Updated — time_zone + time_zone_kolkata</t>
         </is>
       </c>
     </row>
@@ -3614,7 +3531,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST: HTTPS .deb download — can installedCertificateName + installedCertificateType from GET /cloud/certificates be used (types server/client/app), or must trust use CA store / inline PEM? Until confirmed prefer SFTP+BASIC installUserapp.json; do not finalize installUserapp_pinned_ca.json. Details: operation_examples/cloud-apps-install/NEED_LIVE_TEST.md</t>
+          <t>NEED LIVE TEST: HTTPS install with BASIC + installedCertificateType/Name. Draft: installUserapp.json.</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
@@ -3641,7 +3558,7 @@
       </c>
       <c r="P37" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — installed certs for HTTPS install</t>
+          <t>NEED LIVE TEST — installed cert HTTPS app install</t>
         </is>
       </c>
       <c r="Q37" s="4" t="inlineStr">
@@ -3651,7 +3568,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — installedCertificateName/Type vs CA store</t>
+          <t>NEED LIVE TEST — apps/install installed cert</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3695,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST: PFX install via url + type (client/server/app); NONE vs BASIC auth; pfxPassword; success response shape; verify appears on GET /cloud/certificates. Draft packs under cloud-certificates/PUT/ — not finalized. Details: operation_examples/cloud-certificates/NEED_LIVE_TEST.md</t>
+          <t>UPDATED by review: kept old updateCertificate (BASIC client PFX) only; removed newer variants.</t>
         </is>
       </c>
       <c r="J39" s="4" t="n">
@@ -3805,7 +3722,7 @@
       </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — certificate install/update on reader</t>
+          <t>Reviewed — examples ready (old style)</t>
         </is>
       </c>
       <c r="Q39" s="4" t="inlineStr">
@@ -3815,7 +3732,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — PUT certificates (PFX install)</t>
+          <t>Updated — updateCertificate (old)</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3777,7 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — do later. Complex cloud endpoint config (many named variants). Resume after simpler Tier 3 items or when ready for full cloudConfig review.</t>
+          <t>UPDATED by review: 10 examples — all-channel mqtt/tls/aws/azure; data tcp/ws/httpPost; management_event_mqtt; clear_data; data_mqtt_tls_installed_cert.</t>
         </is>
       </c>
       <c r="J40" s="4" t="n">
@@ -3887,7 +3804,7 @@
       </c>
       <c r="P40" s="4" t="inlineStr">
         <is>
-          <t>Deferred — do later</t>
+          <t>Reviewed — 10 cloudConfig examples</t>
         </is>
       </c>
       <c r="Q40" s="4" t="inlineStr">
@@ -3897,7 +3814,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Deferred — do later</t>
+          <t>Updated — 10 examples (+ management_event_mqtt)</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4023,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST: HTTPS firmware download — installedCertificateName/Type (from GET /cloud/certificates) vs inline/file CA (CACertificateFileContent / CACertificateFileLocation)? Same open question as PUT /cloud/apps/install. Until confirmed do not finalize os_https_pinned_ca.json; prefer os/os_basic_auth/os_scp. Details: operation_examples/cloud-os/NEED_LIVE_TEST.md</t>
+          <t>NEED LIVE TEST: HTTPS OS update with installedCertificateType/Name (server / reader-server-cert). Draft pack: os.json.</t>
         </is>
       </c>
       <c r="J43" s="4" t="n">
@@ -4133,7 +4050,7 @@
       </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — installed cert vs inline CA for HTTPS OS update</t>
+          <t>NEED LIVE TEST — installed cert HTTPS OS update</t>
         </is>
       </c>
       <c r="Q43" s="4" t="inlineStr">
@@ -4143,7 +4060,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — installedCertificate vs inline CA (HTTPS OS)</t>
+          <t>NEED LIVE TEST — os installed cert</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4105,7 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Has 2 named request examples — good coverage; MISSING response example (schema declares JSON); Ready in grok-examples: +1 request, +1 response PROPOSED file(s)</t>
+          <t>UPDATED by review: removed response-shaped request body; added RC status reply response. Requests: status, passthru.</t>
         </is>
       </c>
       <c r="J44" s="4" t="n">
@@ -4215,12 +4132,17 @@
       </c>
       <c r="P44" s="4" t="inlineStr">
         <is>
-          <t>Add named variants (mode types / cloud targets / auth)</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q44" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-pass-through/PUT/request.set_passthru_version.json, response.200.rc_status.json</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Updated — status/passthru request + success response</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4326,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>/cloud/ble-config</t>
+          <t>/cloud/bleConfig</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -4419,7 +4341,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: path corrected to /cloud/bleConfig (was ble-config).</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
@@ -4446,12 +4368,17 @@
       </c>
       <c r="P47" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — path corrected to bleConfig</t>
         </is>
       </c>
       <c r="Q47" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-ble-config/GET/response.200.disabled.json</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Updated — path /cloud/bleConfig</t>
         </is>
       </c>
     </row>
@@ -4481,7 +4408,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>/cloud/ble-config</t>
+          <t>/cloud/bleConfig</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -4496,7 +4423,7 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>Has 5 named request examples — good coverage; No JSON response body declared (nothing to exemplify); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: path corrected to /cloud/bleConfig (was ble-config).</t>
         </is>
       </c>
       <c r="J48" s="4" t="n">
@@ -4523,12 +4450,17 @@
       </c>
       <c r="P48" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — path corrected to bleConfig</t>
         </is>
       </c>
       <c r="Q48" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Updated — path /cloud/bleConfig</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4505,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example (get_CACertificates); Audit: keep as-is / already effective</t>
+          <t>DISCUSS with Mayur — GET/PUT/DELETE caCertificates.</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
@@ -4600,12 +4532,17 @@
       </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
       <c r="Q49" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4587,7 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J50" s="4" t="n">
@@ -4677,12 +4614,17 @@
       </c>
       <c r="P50" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q50" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4669,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>Has 12 named request examples — good coverage; Response is empty-string on success; no example (low value); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: single PUT example (config) — MQTT data endpoint.</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
@@ -4754,12 +4696,17 @@
       </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q51" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Updated — one MQTT config example</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4751,7 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Has 3 named request examples — good coverage; Response is empty-string on success; no example (low value); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: Applies To FXR90 only (not FXR60).</t>
         </is>
       </c>
       <c r="J52" s="4" t="n">
@@ -4831,12 +4778,17 @@
       </c>
       <c r="P52" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — FXR90 only</t>
         </is>
       </c>
       <c r="Q52" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Updated — FXR90 only</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4833,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>Has 6 response examples — good coverage; Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J53" s="4" t="n">
@@ -4908,12 +4860,17 @@
       </c>
       <c r="P53" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q53" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4915,7 @@
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>Has 12 named request examples — good coverage; Response is empty-string on success; no example (low value); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J54" s="4" t="n">
@@ -4985,12 +4942,17 @@
       </c>
       <c r="P54" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q54" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5228,7 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example (application/json); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: two examples — fxr60 (no wan0) and fxr90 (includes wan0).</t>
         </is>
       </c>
       <c r="J58" s="4" t="n">
@@ -5293,12 +5255,17 @@
       </c>
       <c r="P58" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q58" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Updated — fxr60 + fxr90 interfaces</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5310,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>Has 2 named request examples — good coverage; Response is empty-string on success; no example (low value); Ready in grok-examples: +1 request, +0 response PROPOSED file(s); Audit: keep as-is / already effective</t>
+          <t>DISCUSS with Mayur / Dhavnesh before finalizing examples.</t>
         </is>
       </c>
       <c r="J59" s="4" t="n">
@@ -5370,12 +5337,17 @@
       </c>
       <c r="P59" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Discuss with Mayur/Dhavnesh</t>
         </is>
       </c>
       <c r="Q59" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-ntpserver/PUT/request.set_ntpServer_single.json</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Discuss with Mayur/Dhavnesh</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5392,7 @@
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J60" s="4" t="n">
@@ -5447,12 +5419,17 @@
       </c>
       <c r="P60" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q60" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5474,7 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J61" s="4" t="n">
@@ -5524,12 +5501,17 @@
       </c>
       <c r="P61" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q61" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5556,7 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example (multiple_values); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: single GET example (region) — Canada / CANADA_FCC_15 live data.</t>
         </is>
       </c>
       <c r="J62" s="4" t="n">
@@ -5601,12 +5583,17 @@
       </c>
       <c r="P62" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q62" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-region/GET/response.200.india.json</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Updated — one region GET (Canada)</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5638,7 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Has 6 named request examples — good coverage; No JSON response body declared (nothing to exemplify); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J63" s="4" t="n">
@@ -5678,12 +5665,17 @@
       </c>
       <c r="P63" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q63" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5720,7 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: single GET example (status).</t>
         </is>
       </c>
       <c r="J64" s="4" t="n">
@@ -5755,12 +5747,17 @@
       </c>
       <c r="P64" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q64" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-status/GET/response.200.running.json</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Updated — one status example</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5879,7 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J66" s="4" t="n">
@@ -5909,12 +5906,17 @@
       </c>
       <c r="P66" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q66" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -5959,7 +5961,7 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective; Path/query params lack examples (query:region)</t>
+          <t>UPDATED by review: live-tested — good.</t>
         </is>
       </c>
       <c r="J67" s="4" t="n">
@@ -5986,12 +5988,17 @@
       </c>
       <c r="P67" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q67" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6043,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>Has 2 named request examples — good coverage; Response is empty-string on success; no example (low value); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: renamed examples to set_password / set_password_rfidadm.</t>
         </is>
       </c>
       <c r="J68" s="4" t="n">
@@ -6063,12 +6070,17 @@
       </c>
       <c r="P68" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q68" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Updated — set_password, set_password_rfidadm</t>
         </is>
       </c>
     </row>
@@ -6113,7 +6125,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: single GET example (version) from live FXR60 response.</t>
         </is>
       </c>
       <c r="J69" s="4" t="n">
@@ -6140,12 +6152,17 @@
       </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q69" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Updated — version from live reader</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6207,7 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>Has 1 response example ((inline)); Audit: keep as-is / already effective</t>
+          <t>UPDATED by review: live availableWifiNetworks scan list (wifi_networks).</t>
         </is>
       </c>
       <c r="J70" s="4" t="n">
@@ -6217,12 +6234,17 @@
       </c>
       <c r="P70" s="4" t="inlineStr">
         <is>
-          <t>No change — leave current examples</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q70" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Updated — live wifi_networks</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6289,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>Has 1 request example (set_startUserapp); Response is empty-string on success; no example (low value); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Path/query params lack examples (path:appname)</t>
+          <t>UPDATED by review: no request body — appname path parameter only; success empty string.</t>
         </is>
       </c>
       <c r="J71" s="4" t="n">
@@ -6294,12 +6316,17 @@
       </c>
       <c r="P71" s="4" t="inlineStr">
         <is>
-          <t>Optional: example "" for success; skip if busy</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q71" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-apps-appname-start/PUT/response.200.success.json</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Updated — no body; path appname only</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6371,7 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>Has 1 request example (set_stopUserapp); Response is empty-string on success; no example (low value); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Path/query params lack examples (path:appname)</t>
+          <t>UPDATED by review: no request body — appname path parameter only; success empty string.</t>
         </is>
       </c>
       <c r="J72" s="4" t="n">
@@ -6371,12 +6398,17 @@
       </c>
       <c r="P72" s="4" t="inlineStr">
         <is>
-          <t>Optional: example "" for success; skip if busy</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q72" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-apps-appname-stop/PUT/response.200.success.json</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Updated — no body; path appname only</t>
         </is>
       </c>
     </row>
@@ -6421,7 +6453,7 @@
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>Has 1 request example (set_uninstallUserapp); Response is empty-string on success; no example (low value); Ready in grok-examples: +0 request, +1 response PROPOSED file(s); Path/query params lack examples (path:appname)</t>
+          <t>UPDATED by review: no request body — appname path parameter only; success empty string.</t>
         </is>
       </c>
       <c r="J73" s="4" t="n">
@@ -6448,12 +6480,17 @@
       </c>
       <c r="P73" s="4" t="inlineStr">
         <is>
-          <t>Optional: example "" for success; skip if busy</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q73" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-apps-appname-uninstall/PUT/response.200.success.json</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Updated — no body; path appname only</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6535,7 @@
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>Spec: REST name is path {caname}; body needs content only. Schema also has optional name (MQTT). NEED LIVE TEST: confirm reader ignores body name and uses path only; also confirm empty-string success. Draft files: InstallCACertificate.json (content only) vs InstallCACertificate_named.json (name+content, MQTT-style).</t>
+          <t>DISCUSS with Mayur — GET/PUT/DELETE caCertificates.</t>
         </is>
       </c>
       <c r="J74" s="4" t="n">
@@ -6525,7 +6562,7 @@
       </c>
       <c r="P74" s="4" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST: path {caname} vs body name; empty-string success</t>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
       <c r="Q74" s="4" t="inlineStr">
@@ -6535,7 +6572,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>NEED LIVE TEST — path vs name (PUT not fully reviewed yet)</t>
+          <t>Discuss with Mayur</t>
         </is>
       </c>
     </row>
@@ -6580,7 +6617,7 @@
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>Has 1 request example (set_refreshCertificate_server); Response is empty-string on success; no example (low value); Ready in grok-examples: +1 request, +0 response PROPOSED file(s); Path/query params lack examples (path:certname)</t>
+          <t>UPDATED by review: refresh — good.</t>
         </is>
       </c>
       <c r="J75" s="4" t="n">
@@ -6607,12 +6644,17 @@
       </c>
       <c r="P75" s="4" t="inlineStr">
         <is>
-          <t>Optional: example "" for success; skip if busy</t>
+          <t>Reviewed — good</t>
         </is>
       </c>
       <c r="Q75" s="4" t="inlineStr">
         <is>
           <t>grok-examples/cloud-certificates-certname/PUT/request.set_refreshCertificate_client.json</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Updated — good</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6776,7 @@
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>Has 1 request example (set_dataToRG); Response is empty-string on success; no example (low value); Empty {} is intentional per schema — document, don't invent fields</t>
+          <t>NEED TO WORK — not finalized.</t>
         </is>
       </c>
       <c r="J77" s="4" t="n">
@@ -6761,12 +6803,17 @@
       </c>
       <c r="P77" s="4" t="inlineStr">
         <is>
-          <t>Optional: example "" for success; skip if busy</t>
+          <t>Need to work</t>
         </is>
       </c>
       <c r="Q77" s="4" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Need to work</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand cloud config and mode example packs; document FXR90-only product notes.
Add 11 PUT /cloud/config and 11 PUT /cloud/mode examples (REST+MQTT), refresh OpenAPI builds, mark eSimConfig/wan0 product notes in operation descriptions, and add FXR90-Pending-Problems.xlsx tracker.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/FXR90-Examples-Effort-Effectiveness.xlsx
+++ b/FXR90-Examples-Effort-Effectiveness.xlsx
@@ -774,6 +774,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="43.2" customHeight="1" s="12">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -907,7 +908,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — do later. Finalize a good GET setting example after PUT settles.</t>
+          <t>DEFERRED — work later (after other endpoints). PUT pack is done (11 examples).</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
@@ -944,7 +945,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Deferred — do later (good setting)</t>
+          <t>Deferred — do later</t>
         </is>
       </c>
     </row>
@@ -3777,7 +3778,7 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: 10 examples — all-channel mqtt/tls/aws/azure; data tcp/ws/httpPost; management_event_mqtt; clear_data; data_mqtt_tls_installed_cert.</t>
+          <t>UPDATED by review: 11 examples — standalone management_cmd_mqtt and management_event_mqtt (two management channels).</t>
         </is>
       </c>
       <c r="J40" s="4" t="n">
@@ -3804,7 +3805,7 @@
       </c>
       <c r="P40" s="4" t="inlineStr">
         <is>
-          <t>Reviewed — 10 cloudConfig examples</t>
+          <t>Reviewed — 11 cloudConfig examples</t>
         </is>
       </c>
       <c r="Q40" s="4" t="inlineStr">
@@ -3814,7 +3815,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Updated — 10 examples (+ management_event_mqtt)</t>
+          <t>Updated — 11 examples (+ management_cmd + management_event)</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3860,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — do later. Many mode variants (SIMPLE/PORTAL/INVENTORY/etc). Resume GET + PUT together when ready for mode deep-dive.</t>
+          <t>DEFERRED — GET review later. PUT pack updated (11 examples).</t>
         </is>
       </c>
       <c r="J41" s="4" t="n">
@@ -3896,7 +3897,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Deferred — do later</t>
+          <t>Deferred — GET later; PUT updated</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3907,7 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>3 — Medium complexity</t>
+          <t>4 — Already good</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -3916,7 +3917,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Very high</t>
+          <t>Already delivered</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -3941,18 +3942,18 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>DEFERRED — do later. Many mode variants (SIMPLE/PORTAL/INVENTORY/etc). Resume GET + PUT together when ready for mode deep-dive.</t>
+          <t>UPDATED from mode_testing/PUT_cloud_mode: 11 PUT examples (4 mode types + filter/query/selects/accesses/reportFilter/tagMetaData/radioStop). No rssiFilter/legacy.</t>
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K42" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>set_mode, set_mode_default_FXR90, set_mode_TAG_FOCUS</t>
+          <t>simple_basic, inventory_with_interval, portal_gpi_trigger, conveyor_basic, with_filter_prefix, with_query, with_selects, with_accesses, with_report_filter, with_tag_metadata, with_radio_stop</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
@@ -3968,7 +3969,7 @@
       </c>
       <c r="P42" s="4" t="inlineStr">
         <is>
-          <t>Deferred — do later</t>
+          <t>Reviewed — examples ready</t>
         </is>
       </c>
       <c r="Q42" s="4" t="inlineStr">
@@ -3978,7 +3979,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Deferred — do later</t>
+          <t>Updated — 11 PUT examples from mode_testing</t>
         </is>
       </c>
     </row>
@@ -4669,18 +4670,18 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>UPDATED by review: single PUT example (config) — MQTT data endpoint.</t>
+          <t>UPDATED: 11 PUT examples — 7 data (mqtt full combo + aws/azure/http/tcp/ws + clear) + 4 GPIO-LED (tag/radio, cloud, gpi, conditions). Globals/management folded into data_mqtt.</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K51" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
-          <t>set_config_data_mqtt_async, set_config_data_aws, set_config_data_azure_mqtt, set_config_data_clear, set_config_data_httpPost, set_config_data_mqtt, set_config_data_tcp_ip, set_config_data_websocket, set_config_global_batching, set_config_global_retention, set_config_management_events, set_config_gpio_led</t>
+          <t>data_mqtt, data_aws, data_azure, data_http_post, data_tcpip_server, data_websocket, clear_data, gpio_led_tag_radio, gpio_led_cloud, gpio_led_gpi, gpio_led_conditions</t>
         </is>
       </c>
       <c r="M51" s="4" t="inlineStr">
@@ -4706,7 +4707,7 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Updated — one MQTT config example</t>
+          <t>Updated — 11 PUT examples (7 data + 4 GPIO-LED)</t>
         </is>
       </c>
     </row>

</xml_diff>